<commit_message>
Arreglo de columnas a excluir
</commit_message>
<xml_diff>
--- a/data/config/pan_config.xlsx
+++ b/data/config/pan_config.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="26">
   <si>
     <t xml:space="preserve">iso3</t>
   </si>
@@ -43,6 +43,12 @@
     <t xml:space="preserve">sheet_name</t>
   </si>
   <si>
+    <t xml:space="preserve">prices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unit</t>
+  </si>
+  <si>
     <t xml:space="preserve">PAN</t>
   </si>
   <si>
@@ -59,6 +65,12 @@
   </si>
   <si>
     <t xml:space="preserve">Oferta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrientes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">millones de B/.</t>
   </si>
   <si>
     <t xml:space="preserve">q02</t>
@@ -95,7 +107,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -116,6 +128,11 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -160,12 +177,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -189,37 +210,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -292,7 +313,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.91"/>
@@ -326,350 +347,446 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>2018</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2018</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="G3" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>2018</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>2019</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+      <c r="H5" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>2019</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="H6" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>2019</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="H7" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+      <c r="H8" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="H9" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="H10" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>2021</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+      <c r="H11" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2021</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="H12" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>2021</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="H13" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+      <c r="H14" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="H15" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
+      </c>
+      <c r="H16" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>